<commit_message>
Grievance Template file's component lookup updated
</commit_message>
<xml_diff>
--- a/SSSNP/template/GBVTemplateFile.xlsx
+++ b/SSSNP/template/GBVTemplateFile.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\KIT\KaroothIT\KIT-GIT\SNSOP-MIS\SSSNP\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{016BDD5F-C5E5-4F5C-8951-14A722C24779}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1FC6C11-DFC6-4043-8072-DA91EA61D124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IMPORT" sheetId="2" r:id="rId1"/>
-    <sheet name="LookupLists" sheetId="3" state="hidden" r:id="rId2"/>
+    <sheet name="LookupLists" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
@@ -4282,12 +4282,6 @@
           </x14:formula1>
           <xm:sqref>O2:O1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="SSSNP Beneficiary" prompt="MANDATORY. Choose an option." xr:uid="{6171DE12-E8E0-4455-A702-3831C5FC4B59}">
-          <x14:formula1>
-            <xm:f>LookupLists!$E$2:$E$4</xm:f>
-          </x14:formula1>
-          <xm:sqref>N2:N1048576</xm:sqref>
-        </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Referral Service Recommended" prompt="Insert text." xr:uid="{6E46AF67-0C99-4242-A553-C49146C7A6C2}">
           <x14:formula1>
             <xm:f>LookupLists!$G$2:$G$9</xm:f>
@@ -4330,6 +4324,12 @@
           </x14:formula1>
           <xm:sqref>L2:L1048576</xm:sqref>
         </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="SNSOP Beneficiary" prompt="MANDATORY. Choose an option." xr:uid="{461ED87D-3F2C-4022-B7EA-0068938AFB7A}">
+          <x14:formula1>
+            <xm:f>LookupLists!$E$2:$E$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>N1:N1048576</xm:sqref>
+        </x14:dataValidation>
       </x14:dataValidations>
     </ext>
   </extLst>

</xml_diff>

<commit_message>
NO added as option for SNSOP Beneficiary dropdown in grievance entries
</commit_message>
<xml_diff>
--- a/SSSNP/template/GBVTemplateFile.xlsx
+++ b/SSSNP/template/GBVTemplateFile.xlsx
@@ -8,20 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\KIT\KaroothIT\KIT-GIT\SNSOP-MIS\SSSNP\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1FC6C11-DFC6-4043-8072-DA91EA61D124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58BC5076-699A-432B-A663-A5EE7815C7D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IMPORT" sheetId="2" r:id="rId1"/>
-    <sheet name="LookupLists" sheetId="3" r:id="rId2"/>
+    <sheet name="LookupLists" sheetId="3" state="hidden" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="67">
   <si>
     <t>Female</t>
   </si>
@@ -219,6 +219,9 @@
   </si>
   <si>
     <t>SNSOP Beneficiary</t>
+  </si>
+  <si>
+    <t>NO</t>
   </si>
 </sst>
 </file>
@@ -4326,7 +4329,7 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="SNSOP Beneficiary" prompt="MANDATORY. Choose an option." xr:uid="{461ED87D-3F2C-4022-B7EA-0068938AFB7A}">
           <x14:formula1>
-            <xm:f>LookupLists!$E$2:$E$3</xm:f>
+            <xm:f>LookupLists!$E$2:$E$4</xm:f>
           </x14:formula1>
           <xm:sqref>N1:N1048576</xm:sqref>
         </x14:dataValidation>
@@ -4421,7 +4424,9 @@
       <c r="A4" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="2"/>
+      <c r="E4" s="2" t="s">
+        <v>66</v>
+      </c>
       <c r="G4" t="s">
         <v>54</v>
       </c>

</xml_diff>